<commit_message>
Agents bulky upload added
</commit_message>
<xml_diff>
--- a/bulky_upload_files/agents_template.xlsx
+++ b/bulky_upload_files/agents_template.xlsx
@@ -24,10 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="56">
-  <si>
-    <t>user</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="59">
   <si>
     <t>D</t>
   </si>
@@ -74,18 +71,12 @@
     <t>account_status</t>
   </si>
   <si>
-    <t>account_tenure</t>
-  </si>
-  <si>
     <t>department</t>
   </si>
   <si>
     <t>organisation</t>
   </si>
   <si>
-    <t>Emerson</t>
-  </si>
-  <si>
     <t>Dambudzo</t>
   </si>
   <si>
@@ -113,9 +104,6 @@
     <t>2years</t>
   </si>
   <si>
-    <t>Abram</t>
-  </si>
-  <si>
     <t>Neymar</t>
   </si>
   <si>
@@ -192,6 +180,27 @@
   </si>
   <si>
     <t>3years</t>
+  </si>
+  <si>
+    <t>Amerson</t>
+  </si>
+  <si>
+    <t>Ebram</t>
+  </si>
+  <si>
+    <t>contract_type</t>
+  </si>
+  <si>
+    <t>contract_tenure</t>
+  </si>
+  <si>
+    <t>FIXED</t>
+  </si>
+  <si>
+    <t>MNO</t>
+  </si>
+  <si>
+    <t>BUFFER</t>
   </si>
 </sst>
 </file>
@@ -539,36 +548,36 @@
   <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.21875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="9.88671875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.5546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.77734375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13" style="1" customWidth="1"/>
-    <col min="11" max="11" width="12" style="1" customWidth="1"/>
-    <col min="12" max="12" width="22.44140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="13.44140625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21.6640625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="16.6640625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.21875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="15.5546875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="15.77734375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.77734375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="13" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12" style="1" customWidth="1"/>
+    <col min="11" max="11" width="22.44140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13.44140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="21.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="16.6640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="15.21875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="15.5546875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="15.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="14.5546875" style="1" customWidth="1"/>
     <col min="19" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="2" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -610,10 +619,10 @@
         <v>14</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -623,64 +632,64 @@
       <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="1">
-        <v>1</v>
+      <c r="C2" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="1">
+        <v>783382395</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G2" s="3" t="s">
+      <c r="J2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="1">
-        <v>783382395</v>
-      </c>
-      <c r="I2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="L2" s="4">
+        <v>32909</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="4">
-        <v>32909</v>
-      </c>
       <c r="N2" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="1">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>53</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>29</v>
@@ -688,221 +697,221 @@
       <c r="E3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G3" s="3" t="s">
+      <c r="F3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="1">
+        <v>783384395</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H3" s="1">
-        <v>783384395</v>
-      </c>
       <c r="I3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" s="4">
+        <v>25628</v>
+      </c>
+      <c r="M3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M3" s="4">
-        <v>25628</v>
-      </c>
       <c r="N3" s="1" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" s="1">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>26</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="1">
+        <v>783389395</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H4" s="1">
-        <v>783389395</v>
-      </c>
       <c r="I4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="1" t="s">
+      <c r="L4" s="4">
+        <v>35708</v>
+      </c>
+      <c r="M4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="M4" s="4">
-        <v>35708</v>
-      </c>
       <c r="N4" s="1" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="O4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B5" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="1">
-        <v>1</v>
+      <c r="C5" s="1" t="s">
+        <v>27</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="1">
+        <v>783382225</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="1">
-        <v>783382225</v>
-      </c>
       <c r="I5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" s="1" t="s">
+      <c r="L5" s="4">
+        <v>4424</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="M5" s="4">
-        <v>4424</v>
-      </c>
       <c r="N5" s="1" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>24</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B6" s="1">
         <v>1</v>
       </c>
-      <c r="C6" s="1">
-        <v>1</v>
+      <c r="C6" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="1">
+        <v>783335395</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="1">
-        <v>783335395</v>
-      </c>
       <c r="I6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="4">
+        <v>36196</v>
+      </c>
+      <c r="M6" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="M6" s="4">
-        <v>36196</v>
-      </c>
       <c r="N6" s="1" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1"/>
-    <hyperlink ref="G3" r:id="rId2"/>
-    <hyperlink ref="G4" r:id="rId3"/>
-    <hyperlink ref="G5" r:id="rId4"/>
-    <hyperlink ref="G6" r:id="rId5"/>
+    <hyperlink ref="F2" r:id="rId1"/>
+    <hyperlink ref="F3" r:id="rId2"/>
+    <hyperlink ref="F4" r:id="rId3"/>
+    <hyperlink ref="F5" r:id="rId4"/>
+    <hyperlink ref="F6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId6"/>

</xml_diff>

<commit_message>
Added agent_type on resources
</commit_message>
<xml_diff>
--- a/bulky_upload_files/agents_template.xlsx
+++ b/bulky_upload_files/agents_template.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="61">
   <si>
     <t>D</t>
   </si>
@@ -201,6 +201,12 @@
   </si>
   <si>
     <t>BUFFER</t>
+  </si>
+  <si>
+    <t>agent_type</t>
+  </si>
+  <si>
+    <t>VOICE_LVC</t>
   </si>
 </sst>
 </file>
@@ -545,31 +551,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.33203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12" style="1" customWidth="1"/>
-    <col min="11" max="11" width="22.44140625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="13.44140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="21.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="16.6640625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="15.21875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.5546875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="15.77734375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="14.5546875" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="3" width="13.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.88671875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.77734375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12" style="1" customWidth="1"/>
+    <col min="12" max="12" width="22.44140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.6640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="15.21875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="15.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="15.77734375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="14.5546875" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="2" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="2" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -577,55 +584,58 @@
         <v>15</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -633,55 +643,58 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="1">
+      <c r="H2" s="1">
         <v>783382395</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="4">
+      <c r="M2" s="4">
         <v>32909</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="Q2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -689,55 +702,58 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G3" s="1">
+      <c r="H3" s="1">
         <v>783384395</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="L3" s="4">
+      <c r="M3" s="4">
         <v>25628</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>24</v>
       </c>
       <c r="Q3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -745,55 +761,58 @@
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <v>783389395</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L4" s="4">
+      <c r="M4" s="4">
         <v>35708</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="N4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="O4" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="P4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="Q4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -801,55 +820,58 @@
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>783382225</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="L5" s="4">
+      <c r="M5" s="4">
         <v>4424</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="N5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="P5" s="1" t="s">
         <v>24</v>
       </c>
       <c r="Q5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R5" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="R5" s="1" t="s">
+      <c r="S5" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>1</v>
       </c>
@@ -857,61 +879,64 @@
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="1">
+      <c r="H6" s="1">
         <v>783335395</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="L6" s="4">
+      <c r="M6" s="4">
         <v>36196</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="N6" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="P6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="Q6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R6" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="R6" s="1" t="s">
+      <c r="S6" s="1" t="s">
         <v>57</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1"/>
-    <hyperlink ref="F3" r:id="rId2"/>
-    <hyperlink ref="F4" r:id="rId3"/>
-    <hyperlink ref="F5" r:id="rId4"/>
-    <hyperlink ref="F6" r:id="rId5"/>
+    <hyperlink ref="G2" r:id="rId1"/>
+    <hyperlink ref="G3" r:id="rId2"/>
+    <hyperlink ref="G4" r:id="rId3"/>
+    <hyperlink ref="G5" r:id="rId4"/>
+    <hyperlink ref="G6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId6"/>

</xml_diff>